<commit_message>
Updated sheet name for spare parts
</commit_message>
<xml_diff>
--- a/data/Markspen_Engineering_Central_Monitor.backup.xlsx
+++ b/data/Markspen_Engineering_Central_Monitor.backup.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1624" uniqueCount="834">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1639" uniqueCount="836">
   <si>
     <t>Branch</t>
   </si>
@@ -2530,6 +2530,12 @@
   </si>
   <si>
     <t>ghjmnb</t>
+  </si>
+  <si>
+    <t>gfds</t>
+  </si>
+  <si>
+    <t>gfd</t>
   </si>
 </sst>
 </file>
@@ -3323,7 +3329,7 @@
         <v>0</v>
       </c>
       <c r="X3" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="Y3" t="s">
         <v>769</v>
@@ -3823,7 +3829,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:P3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.2" defaultColWidth="8.83203125"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -3941,6 +3947,56 @@
         <v>833</v>
       </c>
     </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>770</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>755</v>
+      </c>
+      <c r="D3" t="s">
+        <v>834</v>
+      </c>
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3" t="s">
+        <v>782</v>
+      </c>
+      <c r="G3" t="s">
+        <v>781</v>
+      </c>
+      <c r="H3" t="s">
+        <v>781</v>
+      </c>
+      <c r="I3" t="s">
+        <v>769</v>
+      </c>
+      <c r="J3" t="s">
+        <v>769</v>
+      </c>
+      <c r="K3" t="s">
+        <v>76</v>
+      </c>
+      <c r="L3" t="s">
+        <v>76</v>
+      </c>
+      <c r="M3" t="s">
+        <v>755</v>
+      </c>
+      <c r="N3" t="s">
+        <v>35</v>
+      </c>
+      <c r="O3" t="s">
+        <v>769</v>
+      </c>
+      <c r="P3" t="s">
+        <v>835</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>

</xml_diff>

<commit_message>
October 25 2026 updates
</commit_message>
<xml_diff>
--- a/data/Markspen_Engineering_Central_Monitor.backup.xlsx
+++ b/data/Markspen_Engineering_Central_Monitor.backup.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="675" windowWidth="34200" windowHeight="19785"/>
+    <workbookView xWindow="0" yWindow="675" windowWidth="34200" windowHeight="19785" firstSheet="6" activeTab="14"/>
   </bookViews>
   <sheets>
     <sheet name="Branches" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1638" uniqueCount="835">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1490" uniqueCount="791">
   <si>
     <t>Branch</t>
   </si>
@@ -2289,93 +2289,9 @@
     <t>Follow-Up Due Date</t>
   </si>
   <si>
-    <t>2026-MPH-0001</t>
-  </si>
-  <si>
-    <t>2026/10/24</t>
-  </si>
-  <si>
-    <t>Customer</t>
-  </si>
-  <si>
-    <t>+94765432123</t>
-  </si>
-  <si>
-    <t>Anuradhapura Factory</t>
-  </si>
-  <si>
-    <t>asd</t>
-  </si>
-  <si>
-    <t>qef</t>
-  </si>
-  <si>
-    <t>ML-123</t>
-  </si>
-  <si>
-    <t>2026/10/31</t>
-  </si>
-  <si>
-    <t>fghj</t>
-  </si>
-  <si>
-    <t>2026/10/30</t>
-  </si>
-  <si>
-    <t>ghjk</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>2026/11/01</t>
-  </si>
-  <si>
-    <t>kjhg</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>2026-MPH-0002</t>
-  </si>
-  <si>
-    <t>axca</t>
-  </si>
-  <si>
-    <t>aca</t>
-  </si>
-  <si>
-    <t>casc</t>
-  </si>
-  <si>
-    <t>ca</t>
-  </si>
-  <si>
-    <t>cad</t>
-  </si>
-  <si>
-    <t>2026/10/27</t>
-  </si>
-  <si>
-    <t>2026/10/25</t>
-  </si>
-  <si>
-    <t>2026/10/29</t>
-  </si>
-  <si>
-    <t>adcac</t>
-  </si>
-  <si>
     <t>Lead Technician</t>
   </si>
   <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Yes</t>
-  </si>
-  <si>
     <t>Visit Id</t>
   </si>
   <si>
@@ -2403,30 +2319,6 @@
     <t>Updated Date</t>
   </si>
   <si>
-    <t>VIS-1270</t>
-  </si>
-  <si>
-    <t>2026/10/24 08:30</t>
-  </si>
-  <si>
-    <t>08:30</t>
-  </si>
-  <si>
-    <t>17:00</t>
-  </si>
-  <si>
-    <t>VIS-2154</t>
-  </si>
-  <si>
-    <t>14:00</t>
-  </si>
-  <si>
-    <t>VISIT-02155</t>
-  </si>
-  <si>
-    <t>09:30</t>
-  </si>
-  <si>
     <t xml:space="preserve">Unit Price </t>
   </si>
   <si>
@@ -2481,18 +2373,6 @@
     <t>Payment Status</t>
   </si>
   <si>
-    <t>EXP-2026-001</t>
-  </si>
-  <si>
-    <t>Ceypetco</t>
-  </si>
-  <si>
-    <t>edfg</t>
-  </si>
-  <si>
-    <t>Not Paid</t>
-  </si>
-  <si>
     <t>Completion Date</t>
   </si>
   <si>
@@ -2521,18 +2401,6 @@
   </si>
   <si>
     <t>Remarks</t>
-  </si>
-  <si>
-    <t>dfghj</t>
-  </si>
-  <si>
-    <t>ghjmnb</t>
-  </si>
-  <si>
-    <t>gfds</t>
-  </si>
-  <si>
-    <t>gfd</t>
   </si>
 </sst>
 </file>
@@ -3006,7 +2874,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Y1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -3110,164 +2978,6 @@
         <v>752</v>
       </c>
     </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>753</v>
-      </c>
-      <c r="B2" t="s">
-        <v>754</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>755</v>
-      </c>
-      <c r="F2" t="s">
-        <v>756</v>
-      </c>
-      <c r="G2" t="s">
-        <v>757</v>
-      </c>
-      <c r="H2" t="s">
-        <v>758</v>
-      </c>
-      <c r="I2" t="s">
-        <v>759</v>
-      </c>
-      <c r="J2" t="s">
-        <v>760</v>
-      </c>
-      <c r="K2" t="s">
-        <v>761</v>
-      </c>
-      <c r="L2" t="s">
-        <v>762</v>
-      </c>
-      <c r="M2" t="s">
-        <v>763</v>
-      </c>
-      <c r="N2" t="s">
-        <v>764</v>
-      </c>
-      <c r="O2" t="s">
-        <v>765</v>
-      </c>
-      <c r="P2" t="s">
-        <v>766</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>767</v>
-      </c>
-      <c r="R2" t="s">
-        <v>96</v>
-      </c>
-      <c r="S2" t="s">
-        <v>79</v>
-      </c>
-      <c r="T2" t="s">
-        <v>80</v>
-      </c>
-      <c r="U2" t="s">
-        <v>754</v>
-      </c>
-      <c r="V2">
-        <f>IF(OR(ISBLANK(B2),TRIM(LOWER(X2))="completed",TRIM(LOWER(X2))="invalid",TRIM(LOWER(X2))="cancelled"),0,MAX(0,TODAY()-B2))</f>
-        <v>0</v>
-      </c>
-      <c r="W2">
-        <f>IF(OR(ISBLANK(P2),TRIM(LOWER(X2))="completed",TRIM(LOWER(X2))="invalid",TRIM(LOWER(X2))="cancelled"),0,MAX(0,TODAY()-P2))</f>
-        <v>0</v>
-      </c>
-      <c r="X2" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>768</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>769</v>
-      </c>
-      <c r="B3" t="s">
-        <v>754</v>
-      </c>
-      <c r="C3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
-        <v>770</v>
-      </c>
-      <c r="F3" t="s">
-        <v>771</v>
-      </c>
-      <c r="G3" t="s">
-        <v>772</v>
-      </c>
-      <c r="H3" t="s">
-        <v>773</v>
-      </c>
-      <c r="I3" t="s">
-        <v>774</v>
-      </c>
-      <c r="J3" t="s">
-        <v>774</v>
-      </c>
-      <c r="K3" t="s">
-        <v>775</v>
-      </c>
-      <c r="L3" t="s">
-        <v>774</v>
-      </c>
-      <c r="M3" t="s">
-        <v>776</v>
-      </c>
-      <c r="N3" t="s">
-        <v>774</v>
-      </c>
-      <c r="O3" t="s">
-        <v>765</v>
-      </c>
-      <c r="P3" t="s">
-        <v>777</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>778</v>
-      </c>
-      <c r="R3" t="s">
-        <v>96</v>
-      </c>
-      <c r="S3" t="s">
-        <v>79</v>
-      </c>
-      <c r="T3" t="s">
-        <v>80</v>
-      </c>
-      <c r="U3" t="s">
-        <v>754</v>
-      </c>
-      <c r="V3">
-        <f>IF(OR(ISBLANK(B3),TRIM(LOWER(X3))="completed",TRIM(LOWER(X3))="invalid",TRIM(LOWER(X3))="cancelled"),0,MAX(0,TODAY()-B3))</f>
-        <v>0</v>
-      </c>
-      <c r="W3">
-        <f>IF(OR(ISBLANK(P3),TRIM(LOWER(X3))="completed",TRIM(LOWER(X3))="invalid",TRIM(LOWER(X3))="cancelled"),0,MAX(0,TODAY()-P3))</f>
-        <v>0</v>
-      </c>
-      <c r="X3" t="s">
-        <v>34</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>768</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
@@ -3276,7 +2986,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -3294,63 +3004,7 @@
         <v>37</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>779</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
         <v>753</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D2" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>753</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" t="s">
-        <v>781</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>769</v>
-      </c>
-      <c r="B4" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" t="s">
-        <v>780</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>769</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
-        <v>43</v>
-      </c>
-      <c r="D5" t="s">
-        <v>780</v>
       </c>
     </row>
   </sheetData>
@@ -3361,7 +3015,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O4"/>
+  <dimension ref="A1:O1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -3380,7 +3034,7 @@
   <sheetData>
     <row r="1" spans="1:15" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>782</v>
+        <v>754</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>733</v>
@@ -3392,25 +3046,25 @@
         <v>37</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>783</v>
+        <v>755</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>784</v>
+        <v>756</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>785</v>
+        <v>757</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>786</v>
+        <v>758</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>787</v>
+        <v>759</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>788</v>
+        <v>760</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>789</v>
+        <v>761</v>
       </c>
       <c r="L1" s="10" t="s">
         <v>81</v>
@@ -3422,148 +3076,7 @@
         <v>106</v>
       </c>
       <c r="O1" s="10" t="s">
-        <v>790</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>791</v>
-      </c>
-      <c r="B2" t="s">
-        <v>753</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" t="s">
-        <v>754</v>
-      </c>
-      <c r="F2" t="s">
-        <v>792</v>
-      </c>
-      <c r="G2" t="s">
-        <v>793</v>
-      </c>
-      <c r="H2" t="s">
-        <v>794</v>
-      </c>
-      <c r="I2">
-        <v>8.5</v>
-      </c>
-      <c r="J2" t="s">
-        <v>768</v>
-      </c>
-      <c r="K2" t="s">
-        <v>768</v>
-      </c>
-      <c r="L2" t="s">
-        <v>80</v>
-      </c>
-      <c r="M2" t="s">
-        <v>105</v>
-      </c>
-      <c r="N2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O2" t="s">
-        <v>754</v>
-      </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>795</v>
-      </c>
-      <c r="B3" t="s">
-        <v>753</v>
-      </c>
-      <c r="C3" t="s">
-        <v>2</v>
-      </c>
-      <c r="D3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E3" t="s">
-        <v>754</v>
-      </c>
-      <c r="F3" t="s">
-        <v>792</v>
-      </c>
-      <c r="G3" t="s">
-        <v>793</v>
-      </c>
-      <c r="H3" t="s">
-        <v>796</v>
-      </c>
-      <c r="I3">
-        <v>5.5</v>
-      </c>
-      <c r="J3" t="s">
-        <v>768</v>
-      </c>
-      <c r="K3" t="s">
-        <v>768</v>
-      </c>
-      <c r="L3" t="s">
-        <v>80</v>
-      </c>
-      <c r="M3" t="s">
-        <v>105</v>
-      </c>
-      <c r="N3" t="s">
-        <v>108</v>
-      </c>
-      <c r="O3" t="s">
-        <v>754</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>797</v>
-      </c>
-      <c r="B4" t="s">
-        <v>753</v>
-      </c>
-      <c r="C4" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>754</v>
-      </c>
-      <c r="F4" t="s">
-        <v>792</v>
-      </c>
-      <c r="G4" t="s">
-        <v>793</v>
-      </c>
-      <c r="H4" t="s">
-        <v>798</v>
-      </c>
-      <c r="I4">
-        <v>1</v>
-      </c>
-      <c r="J4" t="s">
-        <v>768</v>
-      </c>
-      <c r="K4" t="s">
-        <v>768</v>
-      </c>
-      <c r="L4" t="s">
-        <v>80</v>
-      </c>
-      <c r="M4" t="s">
-        <v>105</v>
-      </c>
-      <c r="N4" t="s">
-        <v>108</v>
-      </c>
-      <c r="O4" t="s">
-        <v>754</v>
+        <v>762</v>
       </c>
     </row>
   </sheetData>
@@ -3574,7 +3087,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -3595,57 +3108,25 @@
         <v>115</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>799</v>
+        <v>763</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>800</v>
+        <v>764</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>801</v>
+        <v>765</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>802</v>
+        <v>766</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>803</v>
+        <v>767</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>804</v>
+        <v>768</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>753</v>
-      </c>
-      <c r="B2" t="s">
-        <v>120</v>
-      </c>
-      <c r="C2">
-        <v>2450</v>
-      </c>
-      <c r="D2">
-        <v>2</v>
-      </c>
-      <c r="E2">
-        <f>ROUND(C2*D2, 2)</f>
-        <v>4900</v>
-      </c>
-      <c r="F2">
-        <v>15</v>
-      </c>
-      <c r="G2">
-        <f>ROUND(E2-(E2*F2/100), 2)</f>
-        <v>4165</v>
-      </c>
-      <c r="H2">
-        <v>18</v>
-      </c>
-      <c r="I2">
-        <f>ROUND(G2+(G2*H2/100), 2)</f>
-        <v>4914.7</v>
+        <v>769</v>
       </c>
     </row>
   </sheetData>
@@ -3656,7 +3137,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="12" customWidth="1"/>
@@ -3674,84 +3155,43 @@
   <sheetData>
     <row r="1" spans="1:13" s="10" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>806</v>
+        <v>770</v>
       </c>
       <c r="B1" s="10" t="s">
         <v>733</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>807</v>
+        <v>771</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>808</v>
+        <v>772</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>809</v>
+        <v>773</v>
       </c>
       <c r="F1" s="10" t="s">
         <v>17</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>810</v>
+        <v>774</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>811</v>
+        <v>775</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>812</v>
+        <v>776</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>813</v>
+        <v>777</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>814</v>
+        <v>778</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>815</v>
+        <v>779</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>816</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>817</v>
-      </c>
-      <c r="B2" t="s">
-        <v>753</v>
-      </c>
-      <c r="C2" t="s">
-        <v>754</v>
-      </c>
-      <c r="D2" t="s">
-        <v>39</v>
-      </c>
-      <c r="E2" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G2" t="s">
-        <v>762</v>
-      </c>
-      <c r="H2" t="s">
-        <v>818</v>
-      </c>
-      <c r="I2">
-        <v>2500</v>
-      </c>
-      <c r="J2" t="s">
-        <v>819</v>
-      </c>
-      <c r="K2" t="s">
-        <v>79</v>
-      </c>
-      <c r="L2" t="s">
-        <v>96</v>
-      </c>
-      <c r="M2" t="s">
-        <v>820</v>
+        <v>780</v>
       </c>
     </row>
   </sheetData>
@@ -3762,7 +3202,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="12" customWidth="1"/>
@@ -3788,37 +3228,37 @@
         <v>0</v>
       </c>
       <c r="C1" s="10" t="s">
-        <v>821</v>
+        <v>781</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>822</v>
+        <v>782</v>
       </c>
       <c r="E1" s="10" t="s">
-        <v>823</v>
+        <v>783</v>
       </c>
       <c r="F1" s="10" t="s">
-        <v>824</v>
+        <v>784</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>825</v>
+        <v>785</v>
       </c>
       <c r="H1" s="10" t="s">
-        <v>826</v>
+        <v>786</v>
       </c>
       <c r="I1" s="10" t="s">
-        <v>827</v>
+        <v>787</v>
       </c>
       <c r="J1" s="10" t="s">
-        <v>828</v>
+        <v>788</v>
       </c>
       <c r="K1" s="10" t="s">
-        <v>814</v>
+        <v>778</v>
       </c>
       <c r="L1" s="10" t="s">
-        <v>829</v>
+        <v>789</v>
       </c>
       <c r="M1" s="10" t="s">
-        <v>790</v>
+        <v>762</v>
       </c>
       <c r="N1" s="10" t="s">
         <v>27</v>
@@ -3827,107 +3267,7 @@
         <v>752</v>
       </c>
       <c r="P1" s="10" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>753</v>
-      </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2" t="s">
-        <v>754</v>
-      </c>
-      <c r="D2" t="s">
-        <v>831</v>
-      </c>
-      <c r="E2">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>781</v>
-      </c>
-      <c r="G2" t="s">
-        <v>780</v>
-      </c>
-      <c r="H2" t="s">
-        <v>780</v>
-      </c>
-      <c r="I2" t="s">
-        <v>768</v>
-      </c>
-      <c r="J2" t="s">
-        <v>768</v>
-      </c>
-      <c r="K2" t="s">
-        <v>79</v>
-      </c>
-      <c r="L2" t="s">
-        <v>96</v>
-      </c>
-      <c r="M2" t="s">
-        <v>754</v>
-      </c>
-      <c r="N2" t="s">
-        <v>34</v>
-      </c>
-      <c r="O2" t="s">
-        <v>768</v>
-      </c>
-      <c r="P2" t="s">
-        <v>832</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>769</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" t="s">
-        <v>754</v>
-      </c>
-      <c r="D3" t="s">
-        <v>833</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3" t="s">
-        <v>781</v>
-      </c>
-      <c r="G3" t="s">
-        <v>780</v>
-      </c>
-      <c r="H3" t="s">
-        <v>780</v>
-      </c>
-      <c r="I3" t="s">
-        <v>768</v>
-      </c>
-      <c r="J3" t="s">
-        <v>768</v>
-      </c>
-      <c r="K3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L3" t="s">
-        <v>75</v>
-      </c>
-      <c r="M3" t="s">
-        <v>754</v>
-      </c>
-      <c r="N3" t="s">
-        <v>34</v>
-      </c>
-      <c r="O3" t="s">
-        <v>768</v>
-      </c>
-      <c r="P3" t="s">
-        <v>834</v>
+        <v>790</v>
       </c>
     </row>
   </sheetData>

</xml_diff>